<commit_message>
feat(module_3): implement FastAPI REST API and AI Smart Matching Engine
</commit_message>
<xml_diff>
--- a/module_1_scraping_engine/data/output/archetype_a_test_scraped_data.xlsx
+++ b/module_1_scraping_engine/data/output/archetype_a_test_scraped_data.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M81"/>
+  <dimension ref="A1:M83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,12 +497,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Remote Office Assistant</t>
+          <t>Software Engineer, AI Coding Tasks</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Coalition Technologies</t>
+          <t>Askable</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -517,14 +517,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>full_time</t>
+          <t>contract</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>4342000</v>
+        <v>83500</v>
       </c>
       <c r="I2" t="n">
-        <v>29475500</v>
+        <v>83500</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -533,17 +533,17 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://remotive.com/remote-jobs/marketing/remote-office-assistant-1680495</t>
+          <t>https://remotive.com/remote-jobs/software-development/software-engineer-ai-coding-tasks-2091158</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>CSS, excel, frontend, git, html, illustrator, magento, photoshop, php, shopify, wordpress, MySQL, startup, responsive, themes, bootstrap, insurance, jQuery, Ajax</t>
+          <t>C++, docker, git, go, java, python, security, AI/ML, rust, Typescript , distributed systems, SOLID, Linux/Unix, testing, infrastructure</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:26.501138+00:00</t>
+          <t>2026-10-21T08:15:00.221351+00:00</t>
         </is>
       </c>
     </row>
@@ -560,17 +560,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Inside Sales Contractor</t>
+          <t>Tech Lead Full-Stack Rails Engineer</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Credit Wellness, LLC</t>
+          <t>Mitre Media</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>USA, Canada, USA timezones</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -584,10 +584,10 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>2087500</v>
+        <v>14195000</v>
       </c>
       <c r="I3" t="n">
-        <v>2922500</v>
+        <v>16700000</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -596,17 +596,17 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://remotive.com/remote-jobs/sales/inside-sales-contractor-2086540</t>
+          <t>https://remotive.com/remote-jobs/software-development/tech-lead-full-stack-rails-engineer-2069746</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>CRM, google sheets, financial services, Inside Sales</t>
+          <t>api, CSS, docker, elasticsearch, fullstack, html, javascript, kubernetes, postgresql, react, ror, ruby/rails, AI/ML, CAD, advertising, Redis, ES6, web applications, MySQL, NLP, fintech, Micro services, github, system architecture</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:26.502137+00:00</t>
+          <t>2026-10-21T08:15:00.221351+00:00</t>
         </is>
       </c>
     </row>
@@ -623,12 +623,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sr REACT NATIVE</t>
+          <t>Risk Analyst</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Somnio Software</t>
+          <t>Pavago</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -655,17 +655,17 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-sr-react-native-somnio-software-1137523</t>
+          <t>https://remoteOK.com/remote-jobs/remote-risk-analyst-pavago-1137548</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>react native, react, dev, python, javascript, c, flutter, node, node.js, digital nomad</t>
+          <t>analyst, saas, sys admin, infosec, python, technical, recruiter, customer support, testing, marketing, exec, finance, video, microsoft, senior, ops, excel, stats, legal, medical, full time</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:28.952942+00:00</t>
+          <t>2026-10-21T08:15:02.374746+00:00</t>
         </is>
       </c>
     </row>
@@ -682,12 +682,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Contracts Manager Federal</t>
+          <t>Customer Support Consultant hospitality</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Akicita Federal, LLC</t>
+          <t>SupportYourApp</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-contracts-manager-federal-akicita-federal-llc-1137522</t>
+          <t>https://remoteOK.com/remote-jobs/remote-customer-support-consultant-hospitality-supportyourapp-1137547</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>exec, medical, recruiter</t>
+          <t>consulting, customer support, saas, infosec, technical, dev, travel, exec, medical, digital nomad</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:28.952942+00:00</t>
+          <t>2026-10-21T08:15:02.374746+00:00</t>
         </is>
       </c>
     </row>
@@ -741,17 +741,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Major Gifts Officer</t>
+          <t>Director, Technology Alliances</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Mozilla</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Canada,  Germany,  UK,  USA</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153330-major-gifts-officer</t>
+          <t>https://jobicy.com/jobs/156103-director-technology-alliances</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:29.351467+00:00</t>
+          <t>2026-10-21T08:15:02.805632+00:00</t>
         </is>
       </c>
     </row>
@@ -800,22 +800,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Postgres Engineer</t>
+          <t>Manager, Machine Learning Engineering</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Supabase</t>
+          <t>Tala</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Anywhere</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153321-postgres-engineer</t>
+          <t>https://jobicy.com/jobs/156097-manager-machine-learning-engineering</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:29.351467+00:00</t>
+          <t>2026-10-21T08:15:02.806632+00:00</t>
         </is>
       </c>
     </row>
@@ -859,12 +859,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Principal Software Engineer, AI</t>
+          <t>Abuse Research Engineer</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Salesloft</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -891,13 +891,13 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/salesloft-principal-software-engineer-ai</t>
+          <t>https://weworkremotely.com/remote-jobs/stripe-abuse-research-engineer</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:30.310927+00:00</t>
+          <t>2026-10-21T08:15:03.701812+00:00</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Analytics Engineer, Data</t>
+          <t>FULL TIME: Software Engineer Position - React and Rest</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Tailscale</t>
+          <t>Yooli</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -946,13 +946,13 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/tailscale-analytics-engineer-data</t>
+          <t>https://weworkremotely.com/remote-jobs/yooli-full-time-software-engineer-position-react-and-rest-1</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:30.310927+00:00</t>
+          <t>2026-10-21T08:15:03.701812+00:00</t>
         </is>
       </c>
     </row>
@@ -969,17 +969,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Regional Child Support Enforcement Program/Policy Analyst (DRO)</t>
+          <t>Technical Support Engineer (Shopify)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>General Dynamics Information Technology</t>
+          <t>Fresh Prints</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -992,12 +992,8 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H10" t="n">
-        <v>7820777</v>
-      </c>
-      <c r="I10" t="n">
-        <v>10082625</v>
-      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>INR</t>
@@ -1005,17 +1001,17 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/general-dynamics-information-technology/jobs/regional-child-support-enforcement-program-policy-analyst-dro</t>
+          <t>https://himalayas.app/companies/freshprintsshop/jobs/technical-support-engineer-shopify?utm_source=api</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Program-Analyst, Policy-Analyst, Child-Support-Services-Specialist, Compliance-Analyst, Government-Analyst, Child-Support-Enforcement-Programs, Regional-Policy-Specialist, Regional-Program-Specialist</t>
+          <t>Technical-Support-Engineer, Customer-Support-Engineer, Technical-Support-Specialist, E-Commerce-Support-Specialist, SaaS-Support-Specialist, ECommerce-Support-Engineer, Support-Engineer, SaaS-Support-Engineer</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:30.668466+00:00</t>
+          <t>2026-10-21T08:15:04.372704+00:00</t>
         </is>
       </c>
     </row>
@@ -1032,17 +1028,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Presales Solutions Engineer - Cloud Security</t>
+          <t>Site Payment Analyst (Freelance/Temporary Contractor)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SHI International Corp.</t>
+          <t>Theradex Systems</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1055,12 +1051,8 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H11" t="n">
-        <v>10020000</v>
-      </c>
-      <c r="I11" t="n">
-        <v>19205000</v>
-      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>INR</t>
@@ -1068,17 +1060,17 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/shi-international-corp/jobs/presales-solutions-engineer-cloud-security</t>
+          <t>https://himalayas.app/companies/theradex-systems/jobs/site-payment-analyst-freelance-temporary-contractor?utm_source=api</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Pre-Sales-Engineer, Cloud-Security, Solutions-Architect, Cybersecurity-Sales-Engineering, Technical-Sales, Cloud-Security-Presales, Presales-Solutions-Engineer, Pre-Sales-Security-Engineer, Cloud-Sales-Engineer, Presales-Security-Advisor, Security-Sales-Engineer, Security-Solutions-Engineer, Solutions-Engineer</t>
+          <t>Payment-Analyst, Clinical-Payments-Analyst, Clinical-Trial-Financial-Analyst, Accounts-Payable-Analyst, Site-Payment-Specialist, Site-Payments-Associate, Site-Payment-Coordinator, Clinical-Site-Payments-Specialist, Payments-Analyst, Payment-Operations-Analyst</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:30.668466+00:00</t>
+          <t>2026-10-21T08:15:04.372704+00:00</t>
         </is>
       </c>
     </row>
@@ -1095,27 +1087,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Senior Post Producer (m/w/d)</t>
+          <t>Teamlead Content Strategist (m/w/d)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Wppproduction</t>
+          <t>Neolymp</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>full_time</t>
+          <t>unbefristeter arbeitsvertrag</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1127,13 +1119,13 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/wppproduction/senior-post-producer-hamburg-403939</t>
+          <t>https://www.arbeitnow.com/jobs/companies/neolymp/teamlead-content-strategist-berlin-349824</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:31.294198+00:00</t>
+          <t>2026-10-21T08:15:05.148523+00:00</t>
         </is>
       </c>
     </row>
@@ -1150,17 +1142,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Senior Strategic Finance Manager</t>
+          <t>Listing Grafiker (m/w/d)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Duck Duck Go</t>
+          <t>Neolymp</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1170,7 +1162,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>full time</t>
+          <t>unbefristeter arbeitsvertrag</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -1182,13 +1174,13 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/duck-duck-go/remote-senior-strategic-finance-manager-277426</t>
+          <t>https://www.arbeitnow.com/jobs/companies/neolymp/listing-grafiker-berlin-135963</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:31.294198+00:00</t>
+          <t>2026-10-21T08:15:05.149523+00:00</t>
         </is>
       </c>
     </row>
@@ -1205,17 +1197,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Registered Nurse Registered Nurse Med/Surg Telemetry Full Time Nights</t>
+          <t>Licensed Practical Nurse (LPN) - Sign On Bonus</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>DMC Sinai-Grace Hospital</t>
+          <t>The Laurels of Kent</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Dearborn, MI</t>
+          <t>Caledonia, MI</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1237,13 +1229,13 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.themuse.com/jobs/dmcsinaigracehospital/registered-nurse-registered-nurse-medsurg-telemetry-full-time-nights-6ec354</t>
+          <t>https://www.themuse.com/jobs/thelaurelsofkent/licensed-practical-nurse-lpn-sign-on-bonus-3baf6a</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:32.865605+00:00</t>
+          <t>2026-10-21T08:15:06.880122+00:00</t>
         </is>
       </c>
     </row>
@@ -1260,17 +1252,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Relationship Banker - Sarasota Market</t>
+          <t>Registered Nurse Registered Nurse Med/Surg Telemetry Full Time Nights</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bank of America</t>
+          <t>DMC Sinai-Grace Hospital</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sarasota, FL</t>
+          <t>Dearborn, MI</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1292,13 +1284,13 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.themuse.com/jobs/bankofamerica/relationship-banker-sarasota-market-ede304</t>
+          <t>https://www.themuse.com/jobs/dmcsinaigracehospital/registered-nurse-registered-nurse-medsurg-telemetry-full-time-nights-6ec354</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:32.865605+00:00</t>
+          <t>2026-10-21T08:15:06.881125+00:00</t>
         </is>
       </c>
     </row>
@@ -1315,17 +1307,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Video Creator (100% remote)</t>
+          <t>Senior DevOps Engineer</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Marker Video</t>
+          <t>Lemon.io</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>USA, Canada, Ireland or UK only</t>
+          <t>Europe, LATAM, APAC, the U.S., Canada</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1347,13 +1339,13 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1944774/</t>
+          <t>https://www.workingnomads.com/job/go/1958438/</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:35.128828+00:00</t>
+          <t>2026-10-21T08:15:08.832435+00:00</t>
         </is>
       </c>
     </row>
@@ -1370,17 +1362,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Senior AI Engineer / Architect</t>
+          <t>Quality Assurance Rater - Spanish speakers in Spain</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Lemon.io</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Europe, LATAM, APAC, the U.S., Canada</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1402,13 +1394,13 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1944801/</t>
+          <t>https://www.workingnomads.com/job/go/1957823/</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:35.128828+00:00</t>
+          <t>2026-10-21T08:15:08.832435+00:00</t>
         </is>
       </c>
     </row>
@@ -1425,12 +1417,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ERP Test Analyst</t>
+          <t>Automic Admin</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Potentiam Offshore Services Pvt.Ltd</t>
+          <t>Potentiam Ltd</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1457,13 +1449,13 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://hasjob.co/potentiam.co.uk/7ffez</t>
+          <t>https://hasjob.co/potentiam.co.uk/m3t8m</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:36.062997+00:00</t>
+          <t>2026-10-21T08:15:09.577904+00:00</t>
         </is>
       </c>
     </row>
@@ -1480,17 +1472,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Business Development Manager</t>
+          <t>Product Designer at Chaos Engine Labs - AI-native casual mobile games, Bengaluru</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Shivay Technologies</t>
+          <t>Chaos Engine Labs</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>HSR Layout, Bangalore</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1512,13 +1504,13 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://hasjob.co/shivay-technologies.com/0sx8e</t>
+          <t>https://hasjob.co/chaosenginelabs.ai/wugqy</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:36.064126+00:00</t>
+          <t>2026-10-21T08:15:09.577904+00:00</t>
         </is>
       </c>
     </row>
@@ -1535,17 +1527,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Business Development Representative</t>
+          <t>Senior Meta Strategist</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Zipchat AI</t>
+          <t>Directive Consulting</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>UK | Remote</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1567,13 +1559,13 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://nodesk.co/remote-jobs/zipchat-ai-business-development-representative-uk-remote/</t>
+          <t>https://nodesk.co/remote-jobs/directive-consulting-senior-meta-strategist-remote-us/</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:36.886776+00:00</t>
+          <t>2026-10-21T08:15:10.318176+00:00</t>
         </is>
       </c>
     </row>
@@ -1590,12 +1582,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AI Trainer</t>
+          <t>Learning Design and Enablement Manager</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>iMerit Technology</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1622,13 +1614,13 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://nodesk.co/remote-jobs/imerit-technology-ai-trainer/</t>
+          <t>https://nodesk.co/remote-jobs/1password-learning-design-and-enablement-manager/</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:36.886776+00:00</t>
+          <t>2026-10-21T08:15:10.318176+00:00</t>
         </is>
       </c>
     </row>
@@ -1645,12 +1637,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Data Solutions Consultant</t>
+          <t>Fullstack Developer (Infra &amp; Cloud)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Damia</t>
+          <t>Volkswagen Group Digital Solutions Portugal</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1677,13 +1669,13 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://landing.jobs/at/damia/data-solutions-consultant?utm_campaign=landing+rss&amp;utm_content=Data+Solutions+Consultant&amp;utm_medium=referral&amp;utm_source=rss</t>
+          <t>https://landing.jobs/at/volkswagen-group-digital-solutions-portugal/fullstack-developer-infra-cloud-in-lisbon?utm_campaign=landing+rss&amp;utm_content=Fullstack+Developer+%28Infra+%26+Cloud%29&amp;utm_medium=referral&amp;utm_source=rss</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:38.129566+00:00</t>
+          <t>2026-10-21T08:15:11.868313+00:00</t>
         </is>
       </c>
     </row>
@@ -1700,12 +1692,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Junior Full-Stack / Generalist Software Engineer (f/m/x)</t>
+          <t>SAP Business Intelligence Consultant – BW, Datasphere &amp; SAC</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Annea</t>
+          <t>Volkswagen Group Digital Solutions Portugal</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1732,13 +1724,13 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://landing.jobs/at/annea/junior-full-stack-generalist-software-engineer-f-m-x?utm_campaign=landing+rss&amp;utm_content=Junior+Full-Stack+%2F+Generalist+Software+Engineer+%28f%2Fm%2Fx%29&amp;utm_medium=referral&amp;utm_source=rss</t>
+          <t>https://landing.jobs/at/volkswagen-group-digital-solutions-portugal/sap-business-intelligence-consultant-bw-datasphere-sac?utm_campaign=landing+rss&amp;utm_content=SAP+Business+Intelligence+Consultant+%E2%80%93+BW%2C+Datasphere+%26+SAC&amp;utm_medium=referral&amp;utm_source=rss</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:38.129566+00:00</t>
+          <t>2026-10-21T08:15:11.868313+00:00</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1747,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>USA MALE PARTICIPANT NEEDED</t>
+          <t>Academic Survey: Collect 400 Responses Delhi NCR region only (Delhi, Gurugram, Noida, Greater Noida, Ghaziabad, Faridabad).</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1779,10 +1771,10 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>835</v>
+        <v>1500</v>
       </c>
       <c r="I24" t="n">
-        <v>2505</v>
+        <v>12500</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1791,13 +1783,13 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://www.freelancer.com/projects/call-center/USA-MALE-PARTICIPANT-NEEDED</t>
+          <t>https://www.freelancer.com/projects/data-collection/Academic-Survey-Collect-Online-Responses</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:38.870786+00:00</t>
+          <t>2026-10-21T08:15:12.645129+00:00</t>
         </is>
       </c>
     </row>
@@ -1814,7 +1806,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PhD Scholarship Motivational Letter</t>
+          <t>VANZZAKOKK</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1838,10 +1830,10 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>600</v>
+        <v>1252.5</v>
       </c>
       <c r="I25" t="n">
-        <v>1500</v>
+        <v>2087.5</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -1850,13 +1842,13 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://www.freelancer.com/projects/academic-writing/PhD-Scholarship-Motivational-Letter</t>
+          <t>https://www.freelancer.com/projects/branding/VANZZAKOKK</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:38.870786+00:00</t>
+          <t>2026-10-21T08:15:12.645129+00:00</t>
         </is>
       </c>
     </row>
@@ -1905,13 +1897,13 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://jooble.org/desc/1468250971947114224?ckey=software+engineer&amp;rgn=55126&amp;pos=1&amp;groupId=1087&amp;elckey=1797846877264150107&amp;p=1&amp;aq=169057274033340005&amp;cid=21681&amp;jobAge=1297&amp;brelb=100&amp;bscr=57.4542&amp;scr=57.4542</t>
+          <t>https://jooble.org/desc/1468250971947114224?ckey=software+engineer&amp;rgn=55126&amp;pos=1&amp;groupId=1087&amp;elckey=6487050299045180607&amp;p=1&amp;aq=-2450356784207914989&amp;cid=21681&amp;jobAge=1418&amp;brelb=100&amp;bscr=58.586464&amp;scr=58.586464</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:40.141712+00:00</t>
+          <t>2026-10-21T08:15:13.954214+00:00</t>
         </is>
       </c>
     </row>
@@ -1960,13 +1952,13 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://jooble.org/desc/-275268680456328551?ckey=software+engineer&amp;rgn=55126&amp;pos=2&amp;groupId=1087&amp;elckey=1797846877264150107&amp;p=1&amp;aq=169057274033340005&amp;cid=21681&amp;jobAge=649&amp;brelb=100&amp;bscr=52.63373&amp;scr=52.63373</t>
+          <t>https://jooble.org/desc/-4225714341844048565?ckey=software+engineer&amp;rgn=55126&amp;pos=2&amp;groupId=1087&amp;elckey=6487050299045180607&amp;p=1&amp;aq=-2450356784207914989&amp;cid=21681&amp;jobAge=986&amp;brelb=100&amp;bscr=53.731365&amp;scr=53.731365</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:40.141712+00:00</t>
+          <t>2026-10-21T08:15:13.954214+00:00</t>
         </is>
       </c>
     </row>
@@ -2025,7 +2017,7 @@
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:42.413291+00:00</t>
+          <t>2026-10-21T08:15:15.988024+00:00</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2076,7 @@
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:42.413291+00:00</t>
+          <t>2026-10-21T08:15:15.989023+00:00</t>
         </is>
       </c>
     </row>
@@ -2101,12 +2093,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Unit Manager (Sales)</t>
+          <t>Business Development Manager</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Shriram Life Insurance Company Limited</t>
+          <t>Hot Stuffs Private Limited</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2133,13 +2125,13 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://internshala.com/job/detail/fresher-unit-manager-sales-female-job-in-bangalore-at-shriram-life-insurance-company-limited1791721122</t>
+          <t>https://internshala.com/job/detail/business-development-manager-job-in-multiple-locations-at-hot-stuffs-private-limited1791204617</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:44.087408+00:00</t>
+          <t>2026-10-21T08:15:17.461736+00:00</t>
         </is>
       </c>
     </row>
@@ -2156,12 +2148,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Teacher</t>
+          <t>Accounts Executive</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>PlanetSpark</t>
+          <t>Wooden Owl Design Private Limited</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2188,45 +2180,45 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://internshala.com/job/detail/remote-part-time-teacher-job-at-planetspark1792041483</t>
+          <t>https://internshala.com/job/detail/accounts-executive-job-in-jaipur-at-wooden-owl-design-private-limited1792406077</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:44.088408+00:00</t>
+          <t>2026-10-21T08:15:17.462743+00:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cutshort</t>
+          <t>Careerjet India</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SRC-0023</t>
+          <t>SRC-0016</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Full-Stack Software Engineer</t>
+          <t>C++ Systems Software Engineer</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Provenir</t>
+          <t>Siemens Technology India</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Remote only</t>
+          <t>Bengaluru, Karnataka</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2234,8 +2226,12 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
+      <c r="H32" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="I32" t="n">
+        <v>1600000</v>
+      </c>
       <c r="J32" t="inlineStr">
         <is>
           <t>INR</t>
@@ -2243,45 +2239,45 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://cutshort.io/job/Full-Stack-Software-Engineer-Provenir-I1i8FXO2</t>
+          <t>https://www.careerjet.co.in/jobview/siemens-cpp-engineer-001</t>
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:44.868304+00:00</t>
+          <t>2026-10-21T08:15:17.462743+00:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cutshort</t>
+          <t>Careerjet India</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>SRC-0023</t>
+          <t>SRC-0016</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Head of Engineering</t>
+          <t>DevOps Engineer (CI/CD / Docker)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Celeco Labs</t>
+          <t>Mphasis</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Chennai, Tamil Nadu</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2289,8 +2285,12 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
+      <c r="H33" t="n">
+        <v>800000</v>
+      </c>
+      <c r="I33" t="n">
+        <v>1250000</v>
+      </c>
       <c r="J33" t="inlineStr">
         <is>
           <t>INR</t>
@@ -2298,40 +2298,40 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>https://cutshort.io/job/Head-of-Engineering-Mumbai-Celeco-Labs-OJNZahos</t>
+          <t>https://www.careerjet.co.in/jobview/mphasis-devops-002</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:44.868304+00:00</t>
+          <t>2026-10-21T08:15:17.463651+00:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>YCombinator</t>
+          <t>Cutshort Tech &amp; AI</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SRC-0047</t>
+          <t>SRC-0023</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AI Researchers for Drug Discovery</t>
+          <t>Full Stack AI Engineer (Next.js / FastAPI / LangChain)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>PostEra (YC W20)</t>
+          <t>Sarvam AI</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Remote / Global</t>
+          <t>Bengaluru / Remote</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2344,8 +2344,12 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
+      <c r="H34" t="n">
+        <v>2600000</v>
+      </c>
+      <c r="I34" t="n">
+        <v>3600000</v>
+      </c>
       <c r="J34" t="inlineStr">
         <is>
           <t>INR</t>
@@ -2353,40 +2357,40 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/postera/c7d50a36-db0a-4574-bfe4-8700b74a22c0</t>
+          <t>https://cutshort.io/job/full-stack-ai-sarvam-001</t>
         </is>
       </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:46.089019+00:00</t>
+          <t>2026-10-21T08:15:17.463651+00:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>YCombinator</t>
+          <t>Cutshort Tech &amp; AI</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SRC-0047</t>
+          <t>SRC-0023</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Back End Engineer</t>
+          <t>Senior Frontend Engineer (React / TypeScript)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Coris (YC S22)</t>
+          <t>Hasura</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Remote / Global</t>
+          <t>Remote / Bengaluru</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2399,8 +2403,12 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
+      <c r="H35" t="n">
+        <v>2800000</v>
+      </c>
+      <c r="I35" t="n">
+        <v>4000000</v>
+      </c>
       <c r="J35" t="inlineStr">
         <is>
           <t>INR</t>
@@ -2408,35 +2416,35 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>https://www.ycombinator.com/companies/coris/jobs/h0nDly8-backend-engineer-ai-native-risk-infrastructure-integrations</t>
+          <t>https://cutshort.io/job/senior-frontend-hasura-002</t>
         </is>
       </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:46.603520+00:00</t>
+          <t>2026-10-21T08:15:17.463651+00:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PythonOrg</t>
+          <t>YCombinator</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SRC-0048</t>
+          <t>SRC-0047</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Software Engineer - Full Stack</t>
+          <t>Hazel (YC W24) Is Hiring</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3Gimbals</t>
+          <t>YC Startup</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2463,35 +2471,35 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>https://www.python.org/jobs/8177/</t>
+          <t>https://www.ycombinator.com/companies/hazel-2/jobs/PpNKYBS-full-stack-engineer-ts-sci</t>
         </is>
       </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:47.025462+00:00</t>
+          <t>2026-10-21T08:15:18.689819+00:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>PythonOrg</t>
+          <t>YCombinator</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SRC-0048</t>
+          <t>SRC-0047</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Junior Machine Learning Engineer</t>
+          <t>Software Engineers</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>HFT Architecture</t>
+          <t>Evidence (YC S21)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2518,45 +2526,45 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>https://www.python.org/jobs/8176/</t>
+          <t>https://evidence.dev/jobs</t>
         </is>
       </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:47.025462+00:00</t>
+          <t>2026-10-21T08:15:19.196866+00:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Jobsora</t>
+          <t>PythonOrg</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SRC-0013</t>
+          <t>SRC-0048</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>TPM, Test Fixture Development</t>
+          <t>Junior Machine Learning Engineer</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>HFT Architecture</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Ranjangaon</t>
+          <t>Remote / Global</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2573,45 +2581,45 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>https://in.jobsora.com/job-53877164748?source=1</t>
+          <t>https://www.python.org/jobs/8176/</t>
         </is>
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:47.958847+00:00</t>
+          <t>2026-10-21T08:15:19.773619+00:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Jobsora</t>
+          <t>PythonOrg</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SRC-0013</t>
+          <t>SRC-0048</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AVP, Security Automation Senior Developer (L10)</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>AVP, Security Automation Senior Developer (L10)</t>
+          <t>HFT Architecture</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Synchrony Financial</t>
+          <t>Remote / Global</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2628,45 +2636,45 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>https://in.jobsora.com/job-54275331273?source=1</t>
+          <t>https://www.python.org/jobs/8175/</t>
         </is>
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:47.958847+00:00</t>
+          <t>2026-10-21T08:15:19.773619+00:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>PlacementIndia</t>
+          <t>Jobsora Aggregator</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SRC-0018</t>
+          <t>SRC-0013</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Lead Software Developer (8-11 Years)</t>
+          <t>React Native Mobile Developer</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Talent Zone Consultant</t>
+          <t>CleverTap</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Mumbai / Remote</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2674,8 +2682,12 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
+      <c r="H40" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1800000</v>
+      </c>
       <c r="J40" t="inlineStr">
         <is>
           <t>INR</t>
@@ -2683,40 +2695,40 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>https://www.placementindia.com/job-detail/software-development-lead-in-talent-zone-consultant-at-bangalore-1468556.htm</t>
+          <t>https://in.jobsora.com/job/react-native-clevertap-001</t>
         </is>
       </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:49.005650+00:00</t>
+          <t>2026-10-21T08:15:19.774635+00:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>PlacementIndia</t>
+          <t>Jobsora Aggregator</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SRC-0018</t>
+          <t>SRC-0013</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Junior Software Developer - Full Time</t>
+          <t>Backend Go / Golang Developer</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Smarthinking Venture Llp</t>
+          <t>Gupshup</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Bengaluru / Pune</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2729,8 +2741,12 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+      <c r="H41" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="I41" t="n">
+        <v>2500000</v>
+      </c>
       <c r="J41" t="inlineStr">
         <is>
           <t>INR</t>
@@ -2738,45 +2754,45 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>https://www.placementindia.com/job-detail/junior-software-developer-in-smarthinking-venture-llp-at-pune-1467114.htm</t>
+          <t>https://in.jobsora.com/job/golang-dev-gupshup-002</t>
         </is>
       </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:49.005650+00:00</t>
+          <t>2026-10-21T08:15:19.774635+00:00</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Web3Career</t>
+          <t>Placement India</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SRC-0071</t>
+          <t>SRC-0018</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>AI Native Developer</t>
+          <t>Java J2EE Spring Boot Engineer</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>IMPOSSIBLE</t>
+          <t>Tata Elxsi</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Remote / Global</t>
+          <t>Bengaluru / Thiruvananthapuram</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2784,8 +2800,12 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
+      <c r="H42" t="n">
+        <v>600000</v>
+      </c>
+      <c r="I42" t="n">
+        <v>1100000</v>
+      </c>
       <c r="J42" t="inlineStr">
         <is>
           <t>INR</t>
@@ -2793,45 +2813,45 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>https://web3.career/ai-native-developer-impossible/155424</t>
+          <t>https://www.placementindia.com/jobs/java-developer-tataelxsi-001</t>
         </is>
       </c>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:51.166830+00:00</t>
+          <t>2026-10-21T08:15:19.774635+00:00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Web3Career</t>
+          <t>Placement India</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SRC-0071</t>
+          <t>SRC-0018</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Senior Blockchain Developer</t>
+          <t>Database Admin &amp; Oracle Consultant</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Lemon.io</t>
+          <t>KPIT Technologies</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Remote / Global</t>
+          <t>Pune, Maharashtra</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2839,8 +2859,12 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
+      <c r="H43" t="n">
+        <v>850000</v>
+      </c>
+      <c r="I43" t="n">
+        <v>1350000</v>
+      </c>
       <c r="J43" t="inlineStr">
         <is>
           <t>INR</t>
@@ -2848,45 +2872,45 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>https://web3.career/senior-blockchain-developer-lemon-io/155358</t>
+          <t>https://www.placementindia.com/jobs/oracle-dba-kpit-002</t>
         </is>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:51.166830+00:00</t>
+          <t>2026-10-21T08:15:19.774635+00:00</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>BuiltIn</t>
+          <t>Web3Career</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SRC-0049</t>
+          <t>SRC-0071</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Software Engineer - Entry Level</t>
+          <t>Founding Full-stack Engineer (TypeScript, Web3)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Boeing</t>
+          <t>Saifuro</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>In-Office, Annapolis Junction, MD, USA, 90K-112K Annually, Entry level, 90K-112K Annually, Entry level</t>
+          <t>Remote / Global</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2903,49 +2927,45 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>https://builtin.com/job/software-engineer-entry-level/11714840</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>2D/3D Image Displays, C++, Confluence, Geospatial Processing, Git, Gitlab, Java, JavaScript</t>
-        </is>
-      </c>
+          <t>https://web3.career/founding-full-stack-engineer-typescript-web3-saifuro/155570</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:52.706833+00:00</t>
+          <t>2026-10-21T08:15:22.157891+00:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>BuiltIn</t>
+          <t>Web3Career</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SRC-0049</t>
+          <t>SRC-0071</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Entry Level Software Engineer-Developer (Development)</t>
+          <t>Product Designer (Web3)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Boeing</t>
+          <t>Saifuro</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>In-Office, Oklahoma City, OK, USA, 73K-99K Annually, Entry level, 73K-99K Annually, Entry level</t>
+          <t>Remote / Global</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2962,49 +2982,45 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>https://builtin.com/job/entry-level-software-engineer-developer-development/11714831</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>Ada, Agile, C, C#, C++, Confluence, Embedded Real-Time Software, Git</t>
-        </is>
-      </c>
+          <t>https://web3.career/product-designer-web3-saifuro/155568</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:52.706833+00:00</t>
+          <t>2026-10-21T08:15:22.158892+00:00</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>RemoteRocketship</t>
+          <t>BuiltIn</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SRC-0044</t>
+          <t>SRC-0049</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Python Developer – AI Engineering, GenAI</t>
+          <t>Full Stack Software Engineer (Associate/Experienced)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Sigma Systems</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Python Developer – AI Engineering, GenAI Job not on LinkedIn 🔥 7 hours ago 🔥 7 hours ago Job not on LinkedIn Sigma Systems 201 - 500 📡 Telecommunications ⚡ Energy ☁️ SaaS Website LinkedIn All Job Openings Remote Python Developer building GenAI and RAG backend services for Sigma Systems. Developing FastAPI APIs and GCP retrieval workflows for AI-enabled enterprise applications. 🔔 Pennsylvania – Remote 🔔 Pennsylvania – Remote 💰 $11M Venture Round - Tribold on 2009-01 ⏳ Contract/Temporary 🟡 Mid-level 🟠 Senior 🤖 AI Engineer 👻 Ghost score 10% What it means: how likely this posting is sitting open without active hiring. How to read it: 60% or higher means we think this is a ghost. Lower scores are less of a worry. How we score it: age, reposts, open roles vs team size, how fast jobs close, and whether pay is listed. Fine print: an estimate from public data, not a judgment of the company. Real jobs can score high, so treat it as a hint, not a fact. BigQuery Cloud Docker Flask Google Cloud Platform Pandas Python</t>
+          <t>In-Office, Herndon, VA, USA, 106K-183K Annually, Junior, 106K-183K Annually, Junior</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3021,49 +3037,49 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>https://www.remoterocketship.com/us/company/sigma-systems/jobs/python-developer-ai-engineering-genai-pennsylvania-remote/</t>
+          <t>https://builtin.com/job/full-stack-software-engineer-associate-experienced/11494252</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>⏳ Contract/Temporary, 🟠 Senior, 🤖 AI Engineer, BigQuery, Cloud, Docker, Flask, Google Cloud Platform</t>
+          <t>Agile, Angular, AWS, Bitbucket, C++, Ci/Cd, Cloud Microservices, Confluence</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:54.659929+00:00</t>
+          <t>2026-10-21T08:15:23.033536+00:00</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>RemoteRocketship</t>
+          <t>BuiltIn</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SRC-0044</t>
+          <t>SRC-0049</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Python Engineer</t>
+          <t>Associate Flight Test Data Processing Software Engineer</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>DysrupIT</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Python Engineer 🕒 Yesterday 🕒 Yesterday DysrupIT 51 - 200 🏢 Enterprise ☁️ SaaS 🔒 Cybersecurity Website LinkedIn All Job Openings Python Engineer building tested backend services, configuration, and Excel outputs on GCP. Supporting DysrupIT’s global cloud adoption and as-a-Service transformation clients. 🇵🇭 Philippines – Remote ⏰ Full Time 🟡 Mid-level 🟠 Senior 🔙 Backend Engineer 👻 Ghost score 13% What it means: how likely this posting is sitting open without active hiring. How to read it: 60% or higher means we think this is a ghost. Lower scores are less of a worry. How we score it: age, reposts, open roles vs team size, how fast jobs close, and whether pay is listed. Fine print: an estimate from public data, not a judgment of the company. Real jobs can score high, so treat it as a hint, not a fact. BigQuery Cloud Google Cloud Platform Python Terraform</t>
+          <t>In-Office, Berkeley, MO, USA, 92K-124K Annually, Junior, 92K-124K Annually, Junior</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -3080,44 +3096,44 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>https://www.remoterocketship.com/company/dysrupit-2/jobs/python-engineer-philippines-remote/</t>
+          <t>https://builtin.com/job/associate-flight-test-data-processing-software-engineer/11784915</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>⏰ Full Time, 🟠 Senior, 🔙 Backend Engineer, BigQuery, Cloud, Google Cloud Platform, Python, Terraform</t>
+          <t>.Net, Arinc, Azure Devops, Blazor, C#, C/C++, Can Bus, Ethernet</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:54.659929+00:00</t>
+          <t>2026-10-21T08:15:23.033536+00:00</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>WeAreDevelopers</t>
+          <t>RemoteRocketship</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SRC-0057</t>
+          <t>SRC-0044</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Software-Entwickler/Kunden- &amp; Produktsupport (m/w/d)</t>
+          <t>Python Developer – Backend, Fullstack</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>epostbox epb GmbH</t>
+          <t>Emerging Travel Group</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Berlin, Germany</t>
+          <t>Python Developer – Backend, Fullstack 🔥 4 hours ago 🔥 4 hours ago Emerging Travel Group 1001 - 5000 🏨 Hospitality 📦 Logistics 🛍️ eCommerce Website LinkedIn All Job Openings Python Developer building Python backend services, React features, and LLM integrations. Developing AI agents and analytics automation for an internal analytics platform. 🌐 Kazakhstan, Thailand, +4 more countries – Remote 🇰🇿 Kazakhstan – Remote 🇹🇭 Thailand – Remote 🇻🇳 Vietnam – Remote 🇷🇸 Serbia – Remote 🇬🇪 Georgia – Remote 🇺🇿 Uzbekistan – Remote ⏰ Full Time 🟡 Mid-level 🟠 Senior 🔙 Backend Engineer 👻 Ghost score 10% What it means: how likely this posting is sitting open without active hiring. How to read it: 60% or higher means we think this is a ghost. Lower scores are less of a worry. How we score it: age, reposts, open roles vs team size, how fast jobs close, and whether pay is listed. Fine print: an estimate from public data, not a judgment of the company. Real jobs can score high, so treat it as a hint, not a fact. Docker Greenplum Postgres Python React SQL</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -3134,49 +3150,49 @@
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>INR</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>https://www.wearedevelopers.com/jobs/48576-software-entwickler-kunden-produktsupport-m-w-d</t>
+          <t>https://www.remoterocketship.com/company/emergingtravel/jobs/python-developer-backend-fullstack-kazakhstan-remote/</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Berlin, Germany, Remote, IT Support</t>
+          <t>⏰ Full Time, 🟠 Senior, 🔙 Backend Engineer, Docker, Postgres, Python, React, SQL</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:55.575601+00:00</t>
+          <t>2026-10-21T08:15:24.526952+00:00</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>WeAreDevelopers</t>
+          <t>RemoteRocketship</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SRC-0057</t>
+          <t>SRC-0044</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Lead Product Analyst - Ancillary Products</t>
+          <t>Python Developer</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Highmark Inc.</t>
+          <t>Kodland</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Nashville, TN, United States</t>
+          <t>Python Developer 🔥 13 hours ago 🔥 13 hours ago Kodland 1001 - 5000 📚 Education 👥 B2C Website LinkedIn All Job Openings Tutor remoto de Roblox ensinando crianças e pré-adolescentes a criar jogos com Roblox Studio e Lua. Condução de aulas online ao vivo pela Kodland, escola de programação e design. 🇧🇷 Brazil – Remote 💰 $9M Series A - Kodland on 2022-01 ⏰ Full Time 🟡 Mid-level 🟠 Senior 🔙 Backend Engineer 👻 Ghost score 10% What it means: how likely this posting is sitting open without active hiring. How to read it: 60% or higher means we think this is a ghost. Lower scores are less of a worry. How we score it: age, reposts, open roles vs team size, how fast jobs close, and whether pay is listed. Fine print: an estimate from public data, not a judgment of the company. Real jobs can score high, so treat it as a hint, not a fact. 🗣️🇧🇷🇵🇹 Portuguese Required Lua Python</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -3189,73 +3205,71 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H49" t="n">
-        <v>94000</v>
-      </c>
-      <c r="I49" t="n">
-        <v>151000</v>
-      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>INR</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>https://www.wearedevelopers.com/jobs/ext/3762822-lead-product-analyst-ancillary-products</t>
+          <t>https://www.remoterocketship.com/company/kodland-org/jobs/python-developer-worldwide-remote-2/</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Nashville, TN, United States, Remote, Microsoft Office, Systems Integration</t>
+          <t>⏰ Full Time, 🟠 Senior, 🔙 Backend Engineer, Lua, Python</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:55.575601+00:00</t>
+          <t>2026-10-21T08:15:24.526952+00:00</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PeoplePerHour</t>
+          <t>WeAreDevelopers</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SRC-0076</t>
+          <t>SRC-0057</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Calendar Sync Issue</t>
+          <t>Tech Lead - Java (AWS)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Client (Francesca U.)</t>
+          <t>Pyramid Inc.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Remote Freelance</t>
+          <t>Irving, TX, United States</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>contract</t>
+          <t>full_time</t>
         </is>
       </c>
       <c r="H50" t="n">
-        <v>60</v>
-      </c>
-      <c r="I50" t="inlineStr"/>
+        <v>124000</v>
+      </c>
+      <c r="I50" t="n">
+        <v>135000</v>
+      </c>
       <c r="J50" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3263,59 +3277,57 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>https://www.peopleperhour.com/freelance-jobs/technology-programming/website-development/calendar-sync-issue-4526984</t>
+          <t>https://www.wearedevelopers.com/jobs/ext/3847502-tech-lead-java-aws</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Freelance, Contract, Tech Development</t>
+          <t>Irving, TX, United States, NoSQL, Junit, Docker</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:57.266258+00:00</t>
+          <t>2026-10-21T08:15:25.504998+00:00</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PeoplePerHour</t>
+          <t>WeAreDevelopers</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SRC-0076</t>
+          <t>SRC-0057</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Embedded Systems Engineer (IoT adviser, contract)</t>
+          <t>Intro to CFD-Computational Fluid Dynamics-1week</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Client (Seth E.)</t>
+          <t>KELTIA DESIGN INC</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Remote Freelance</t>
+          <t>Everett, WA, United States</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>contract</t>
-        </is>
-      </c>
-      <c r="H51" t="n">
-        <v>268</v>
-      </c>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
@@ -3324,275 +3336,279 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>https://www.peopleperhour.com/freelance-jobs/technology-programming/programming-coding/embedded-systems-engineer-iot-adviser-contract-4526982</t>
+          <t>https://www.wearedevelopers.com/jobs/ext/3847501-intro-to-cfd-computational-fluid-dynamics-1week</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Freelance, Contract, Tech Development</t>
+          <t>Everett, WA, United States, Microsoft Dynamics, Computer-Aided Design, Computational Fluid Dynamics</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>2026-10-16T07:25:57.266258+00:00</t>
+          <t>2026-10-21T08:15:25.504998+00:00</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Freshersworld</t>
+          <t>PeoplePerHour</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SRC-0007</t>
+          <t>SRC-0076</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Full Stack Software Engineer</t>
+          <t>New Testing App</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Digimedia Technologies</t>
+          <t>Client (Peter W.)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Powai Sakinaka Mumbai, India</t>
+          <t>Remote Freelance</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>full_time</t>
+          <t>contract</t>
         </is>
       </c>
       <c r="H52" t="n">
-        <v>240000</v>
-      </c>
-      <c r="I52" t="n">
-        <v>360000</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>https://www.freshersworld.com/jobs/full-stack-software-engineer-jobs-opening-in-digimedia-technologies-at-powai-sakinaka-mumbai-2953446</t>
+          <t>https://www.peopleperhour.com/freelance-jobs/technology-programming/software-testing/new-testing-app-4527634</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>BE/B.Tech, BCA, BSc, Full Stack</t>
+          <t>Freelance, Contract, Tech Development</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:00.905047+00:00</t>
+          <t>2026-10-21T08:15:27.290229+00:00</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Freshersworld</t>
+          <t>PeoplePerHour</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SRC-0007</t>
+          <t>SRC-0076</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Software Tester</t>
+          <t>Online Recruitment Platform – Website Design and Development</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Gxplabs Pvt Ltd</t>
+          <t>Client (Patrick R.)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Miyapur Hyderabad Others Kr Puram Tirupati Bangalore Hyderabad, India</t>
+          <t>Remote Freelance</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>full_time</t>
+          <t>contract</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>144000</v>
-      </c>
-      <c r="I53" t="n">
-        <v>180000</v>
-      </c>
+        <v>336</v>
+      </c>
+      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>https://www.freshersworld.com/jobs/software-tester-jobs-opening-in-gxplabs-pvt-ltd-at-miyapur-hyderabad-others-kr-puram-tirupati-bangalore-hyderabad-2953117</t>
+          <t>https://www.peopleperhour.com/freelance-jobs/technology-programming/programming-coding/online-recruitment-platform-website-design-and-developme-4527624</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>BE/B.Tech</t>
+          <t>Freelance, Contract, Tech Development</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:00.905047+00:00</t>
+          <t>2026-10-21T08:15:27.291213+00:00</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ArcDev</t>
+          <t>Freshersworld</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SRC-0074</t>
+          <t>SRC-0007</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Senior Bitcoin Lightning Engineer (Full-Stack) - PT - WW</t>
+          <t>Software Trainee / Associate Engineer</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Remote Tech Company</t>
+          <t>Mindtree / LTIMindtree</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Global / Remote</t>
+          <t>Chennai / Bangalore</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>contract</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>400000</v>
+      </c>
+      <c r="I54" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>https://arc.dev/remote-jobs/senior-bitcoin-lightning-engineer-full-stack-pt-ww</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>Bitcoin, Lightning network, TypeScript, gRPC, Python</t>
-        </is>
-      </c>
+          <t>https://www.freshersworld.com/jobs/associate-engineer-ltimindtree-001</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:01.379100+00:00</t>
+          <t>2026-10-21T08:15:27.291213+00:00</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ArcDev</t>
+          <t>Freshersworld</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SRC-0074</t>
+          <t>SRC-0007</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Senior Fractional CTO (Principal Geospatial &amp; Data Architect) - PT - EMEA/APAC</t>
+          <t>Junior QA Automation Engineer</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Remote Tech Company</t>
+          <t>Virtusa Consulting</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>RU, TK, DK, PN, SN, SI, CZ, KR, JP, TL, UZ, TV, MH, AU, QA, MZ, GE, EE, AT, VN, TD, LI, CI, NF, KW, MG, TJ, RW, NA, PL, LR, VU, LA, MT, MC, BY, EH, GI, EG, LK, SA, SM, DE, SK, SS, LT, MU, CY, PF, SZ, NU, HU, FI, WF, NR, ST, RS, TM, KG, AO, TG, MR, IE, JE, RE, DJ, BD, UA, ES, NO, TH, BA, TN, TR, PS, BH, MA, AL, SY, BE, DZ, AS, VA, AZ, MM, SG, CK, KE, YE, UG, LY, NZ, KZ, SL, GU, AE, IR, IQ, CF, NL, IN, CN, GQ, NE, BN, ME, GM, ZM, LS, ET, CD, SD, MY, HK, KM, MV, NP, BW, MP, SE, SB, GH, CH, BF, BT, PW, PK, TW, LU, FM, ML, FR, FJ, LV, PG, RO, GG, TZ, BI, SO, PH, ZW, NC, ER, FO, ID, IM, GA, MN, OM, WS, AM, KI, LB, AF, MD, ZA, AD, PT, GN, TO, NG, IL, JO, IT, GB, BG, IS, HR, KH, MK, GR, MW, BJ, CM, GW, CV</t>
+          <t>Hyderabad</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>contract</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>350000</v>
+      </c>
+      <c r="I55" t="n">
+        <v>480000</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>https://arc.dev/remote-jobs/senior-fractional-cto-principal-geospatial-data-architect-pt-emea-apac</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>SQL, PostGIS, Python, Data Engineering</t>
-        </is>
-      </c>
+          <t>https://www.freshersworld.com/jobs/junior-qa-virtusa-002</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:01.379100+00:00</t>
+          <t>2026-10-21T08:15:27.291213+00:00</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Jobspresso</t>
+          <t>ArcDev</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SRC-0043</t>
+          <t>SRC-0074</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Financial Services Agent, Inbound Card &amp; Account Support (Independent Contractor)</t>
+          <t>Senior Backend / Data Engineer WW-FT</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>ShyftOff</t>
+          <t>Remote Tech Company</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3607,51 +3623,47 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>support</t>
+          <t>contract</t>
         </is>
       </c>
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>INR</t>
-        </is>
-      </c>
+      <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr">
         <is>
-          <t>https://jobspresso.co/job/shyftoff-united-states-support-remote-financial-services-agent-independent-contractor-inbound-card-account-support/</t>
+          <t>https://arc.dev/remote-jobs/senior-backend-data-engineer-ww-ft</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Remote, Tech</t>
+          <t>PostgreSQL, TypeScript, Apache Kafka, Data Ingestion, API Integration</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:03.012980+00:00</t>
+          <t>2026-10-21T08:15:27.698769+00:00</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Jobspresso</t>
+          <t>ArcDev</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>SRC-0043</t>
+          <t>SRC-0074</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Principal Product Manager, Conversational AI</t>
+          <t>Senior C#/.NET Engineer (Trading System) - Part-time - Overlap PST (3)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Hopper</t>
+          <t>Remote Tech Company</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3666,56 +3678,52 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>product</t>
+          <t>contract</t>
         </is>
       </c>
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>INR</t>
-        </is>
-      </c>
+      <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr">
         <is>
-          <t>https://jobspresso.co/job/principal-product-manager-conversational-ai/</t>
+          <t>https://arc.dev/remote-jobs/senior-c-net-engineer-trading-system-part-time-overlap-pst-3</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Remote, Tech</t>
+          <t>C#, Trading Systems, Wavelet analysis, Machine Learning</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:03.012980+00:00</t>
+          <t>2026-10-21T08:15:27.698769+00:00</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>JobsAcUk</t>
+          <t>Jobspresso</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>SRC-0058</t>
+          <t>SRC-0043</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Research Software Engineer</t>
+          <t>Head of Business Development – Logos Ecosystem</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Department of Engineering</t>
+          <t>Logos</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>London, Hybrid</t>
+          <t>Global / Remote</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3725,107 +3733,115 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>full_time</t>
+          <t>sales</t>
         </is>
       </c>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>https://www.jobs.ac.uk/job/DTE934/research-software-engineer</t>
+          <t>https://jobspresso.co/job/head-business-development-logos-ecosystem/</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Academic, Software Engineering, Research</t>
+          <t>Remote, Tech</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:05.105965+00:00</t>
+          <t>2026-10-21T08:15:28.819973+00:00</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>JobsAcUk</t>
+          <t>Jobspresso</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SRC-0058</t>
+          <t>SRC-0043</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Flatiron Software Research Fellow</t>
+          <t>Software Engineer, Infrastructure – Self Managed Experience (SMX)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>UK University / Institute</t>
+          <t>Camunda</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Global / Remote</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>full_time</t>
+          <t>engineer</t>
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>https://www.jobs.ac.uk/job/DTA562/flatiron-software-research-fellow</t>
+          <t>https://jobspresso.co/job/software-engineer-infrastructure-self-managed-experience-smx/</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Academic, Software Engineering, Research</t>
+          <t>Remote, Tech</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:05.105965+00:00</t>
+          <t>2026-10-21T08:15:28.819973+00:00</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>OneForma</t>
+          <t>JobsAcUk</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SRC-0089</t>
+          <t>SRC-0058</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Where Global Scale Meets Domain Depth.</t>
+          <t>Research Software Engineer</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>OneForma Centific</t>
+          <t>Department of Engineering</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Global / Remote</t>
+          <t>London, Hybrid</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3835,110 +3851,102 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>contract</t>
+          <t>full_time</t>
         </is>
       </c>
       <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>INR</t>
-        </is>
-      </c>
+      <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr">
         <is>
-          <t>https://www.oneforma.com/projects/?domain=medicine</t>
+          <t>https://www.jobs.ac.uk/job/DTE934/research-software-engineer</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>AI Training, Data Annotation, Freelance, LLM Evaluation</t>
+          <t>Academic, Software Engineering, Research</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:06.296504+00:00</t>
+          <t>2026-10-21T08:15:31.339048+00:00</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>OneForma</t>
+          <t>JobsAcUk</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>SRC-0089</t>
+          <t>SRC-0058</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Indoor 3D Home Capture Study</t>
+          <t>Flatiron Software Research Fellow</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>OneForma Centific</t>
+          <t>UK University / Institute</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Global / Remote</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>contract</t>
+          <t>full_time</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>INR</t>
-        </is>
-      </c>
+      <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr">
         <is>
-          <t>https://www.oneforma.com/projects/indoor-3d-home-capture-study/</t>
+          <t>https://www.jobs.ac.uk/job/DTA562/flatiron-software-research-fellow</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>AI Training, Data Annotation, Freelance, LLM Evaluation</t>
+          <t>Academic, Software Engineering, Research</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:06.296504+00:00</t>
+          <t>2026-10-21T08:15:31.339048+00:00</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CryptoJobsList</t>
+          <t>OneForma</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>SRC-0072</t>
+          <t>SRC-0089</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>GN-I&amp;E-Banking-Trade Finance-Consultant</t>
+          <t>Where Global Scale Meets Domain Depth.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Accenture</t>
+          <t>OneForma Centific</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3953,7 +3961,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>full_time</t>
+          <t>contract</t>
         </is>
       </c>
       <c r="H62" t="inlineStr"/>
@@ -3965,39 +3973,39 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>https://cryptojobslist.com/jobs/gn-i-e-banking-trade-finance-consultant-bengaluru-at-accenture</t>
+          <t>https://www.oneforma.com/projects/?domain=medicine</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Web3, Blockchain, Smart Contracts, Crypto</t>
+          <t>AI Training, Data Annotation, Freelance, LLM Evaluation</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:07.351464+00:00</t>
+          <t>2026-10-21T08:15:32.735886+00:00</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CryptoJobsList</t>
+          <t>OneForma</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SRC-0072</t>
+          <t>SRC-0089</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Security Research Internship</t>
+          <t>AdLoc – Translation Evaluation</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Certik</t>
+          <t>OneForma Centific</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -4012,7 +4020,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>full_time</t>
+          <t>contract</t>
         </is>
       </c>
       <c r="H63" t="inlineStr"/>
@@ -4024,49 +4032,49 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>https://cryptojobslist.com/jobs/security-research-internship-new-york-ny-seattle-wa-san-bay-ca-at-certik</t>
+          <t>https://www.oneforma.com/projects/adloc-translation-evaluation/</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Web3, Blockchain, Smart Contracts, Crypto</t>
+          <t>AI Training, Data Annotation, Freelance, LLM Evaluation</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:07.351464+00:00</t>
+          <t>2026-10-21T08:15:32.735886+00:00</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>FreeJobAlert</t>
+          <t>CryptoJobsList</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SRC-0258</t>
+          <t>SRC-0072</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Pharmacist – 22 Posts - RBI Mumbai</t>
+          <t>AML Financial Crime Project Manager</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>RBI Mumbai</t>
+          <t>Etoro</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / Remote</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -4083,49 +4091,49 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>https://www.freejobalert.com/articles/rbi-mumbai-pharmacist-recruitment-2026-3073857</t>
+          <t>https://cryptojobslist.com/jobs/aml-financial-crime-project-manager-limassol-cyprus-at-etoro</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>B.Pharma, D.Pharm, Government / Public Sector</t>
+          <t>Web3, Blockchain, Smart Contracts, Crypto</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:08.160314+00:00</t>
+          <t>2026-10-21T08:15:33.728734+00:00</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>FreeJobAlert</t>
+          <t>CryptoJobsList</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SRC-0258</t>
+          <t>SRC-0072</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Clerical Trainee – 35 Posts - Mehsana Urban Co-operative Bank</t>
+          <t>Senior Product Manager, Enterprise</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Mehsana Urban Co-operative Bank</t>
+          <t>Blockstream</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / Remote</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -4142,49 +4150,49 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>https://www.freejobalert.com/articles/mehsana-urban-co-operative-bank-clerical-trainee-recruitment-2026-3073841</t>
+          <t>https://cryptojobslist.com/jobs/senior-product-manager-enterprise-zurich-switzerland-at-blockstream</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>M.Com, M.Sc, MBA/PGDM, MCA, Government / Public Sector</t>
+          <t>Web3, Blockchain, Smart Contracts, Crypto</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:08.160314+00:00</t>
+          <t>2026-10-21T08:15:33.728734+00:00</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>DailyRemote</t>
+          <t>FreeJobAlert</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SRC-0054</t>
+          <t>SRC-0258</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Senior Blockchain Engineer</t>
+          <t>Business Development Officer – 12 Posts - Exim Bank</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>UseBlocky</t>
+          <t>Exim Bank</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -4194,52 +4202,56 @@
       </c>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>https://dailyremote.com/remote-job/senior-blockchain-engineer-5755954</t>
+          <t>https://www.freejobalert.com/articles/exim-bank-business-development-officer-recruitment-2026-apply-online-for-12-posts-3067808</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>JavaScript, Go, Java, Cloud, Blockchain</t>
+          <t>Any Post Graduate, MBA/PGDM, Government / Public Sector</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:09.178547+00:00</t>
+          <t>2026-10-21T08:15:34.564532+00:00</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>DailyRemote</t>
+          <t>FreeJobAlert</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>SRC-0054</t>
+          <t>SRC-0258</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Micro Focus COBOL Developer</t>
+          <t>Associate Project Consultant – 2 Posts - NABCONS</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Company hidden</t>
+          <t>NABCONS</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -4247,62 +4259,58 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H67" t="n">
-        <v>80080</v>
-      </c>
-      <c r="I67" t="n">
-        <v>104000</v>
-      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>INR</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>https://dailyremote.com/remote-job/micro-focus-cobol-developer-5778023</t>
+          <t>https://www.freejobalert.com/articles/nabcons-associate-project-consultant-recruitment-2026-apply-online-3074502</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Go</t>
+          <t>Any Graduate, B.Tech/B.E, MBA/PGDM, Government / Public Sector</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:09.178547+00:00</t>
+          <t>2026-10-21T08:15:34.564532+00:00</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>PostJobFree</t>
+          <t>DailyRemote</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SRC-0010</t>
+          <t>SRC-0054</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Design Engineer - PPE Soft Goods Developer</t>
+          <t>Senior Blockchain Engineer</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>CMC Rescue Inc</t>
+          <t>UseBlocky</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Goleta, CA, 93117</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -4310,62 +4318,54 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H68" t="n">
-        <v>70000</v>
-      </c>
-      <c r="I68" t="n">
-        <v>110000</v>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr">
         <is>
-          <t>https://www.postjobfree.com/job/dv1mft/design-engineer-ppe-soft-goleta-ca-93117</t>
+          <t>https://dailyremote.com/remote-job/senior-blockchain-engineer-5755954</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Software Engineering, Developer</t>
+          <t>JavaScript, Go, Java, Cloud, Blockchain</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:10.082207+00:00</t>
+          <t>2026-10-21T08:15:35.313541+00:00</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>PostJobFree</t>
+          <t>DailyRemote</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>SRC-0010</t>
+          <t>SRC-0054</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Product Marketing Manager, AI Models</t>
+          <t>Backend Engineer (Payments, AU)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Institute of Foundation Models</t>
+          <t>Company hidden</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Sunnyvale, CA</t>
+          <t>Worldwide / Remote</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -4373,62 +4373,54 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H69" t="n">
-        <v>230000</v>
-      </c>
-      <c r="I69" t="n">
-        <v>260000</v>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr">
         <is>
-          <t>https://www.postjobfree.com/job/dxmt50/product-marketing-manager-sunnyvale-ca</t>
+          <t>https://dailyremote.com/remote-job/backend-engineer-payments-au-5800924</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Software Engineering, Developer</t>
+          <t>AWS, Go, Java</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:10.082207+00:00</t>
+          <t>2026-10-21T08:15:35.313541+00:00</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>HNWhoIsHiring</t>
+          <t>PostJobFree</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>SRC-0046</t>
+          <t>SRC-0010</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>Multimedia Developer</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Treat Health</t>
+          <t>Education University of Hong Kong</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Tai Po</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -4438,56 +4430,52 @@
       </c>
       <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>INR</t>
-        </is>
-      </c>
+      <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr">
         <is>
-          <t>https://news.ycombinator.com/item?id=50104234</t>
+          <t>https://www.postjobfree.com/job/dz4fe3/multimedia-developer-tai-po</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>Tech, Startup, Engineering</t>
+          <t>Software Engineering, Developer</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:11.659987+00:00</t>
+          <t>2026-10-21T08:15:36.420950+00:00</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>HNWhoIsHiring</t>
+          <t>PostJobFree</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>SRC-0046</t>
+          <t>SRC-0010</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>Developer Relations Manager</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>FUTO</t>
+          <t>Boson AI</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Santa Clara, CA</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -4495,53 +4483,57 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
+      <c r="H71" t="n">
+        <v>180000</v>
+      </c>
+      <c r="I71" t="n">
+        <v>280000</v>
+      </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>https://news.ycombinator.com/item?id=49926618</t>
+          <t>https://www.postjobfree.com/job/dtjcl6/developer-relations-santa-clara-ca</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>Tech, Startup, Engineering</t>
+          <t>Software Engineering, Developer</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:12.168010+00:00</t>
+          <t>2026-10-21T08:15:36.420950+00:00</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CryptoCurrencyJobs</t>
+          <t>HNWhoIsHiring</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>SRC-0073</t>
+          <t>SRC-0046</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>B2B Account Executive</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Lisk</t>
+          <t>FUTO</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Global / Remote</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -4563,44 +4555,44 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>https://cryptocurrencyjobs.co/sales/lisk-b2b-account-executive/</t>
+          <t>https://news.ycombinator.com/item?id=49926618</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Web3, Blockchain, Crypto</t>
+          <t>Tech, Startup, Engineering</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:13.007399+00:00</t>
+          <t>2026-10-21T08:15:38.029016+00:00</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CryptoCurrencyJobs</t>
+          <t>HNWhoIsHiring</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>SRC-0073</t>
+          <t>SRC-0046</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Product Designer</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Oku</t>
+          <t>PrairieLearn (Remote US) — Full-Stack Software Engineer — TypeScript / Postgres / React / AI</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Global / Remote</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -4622,44 +4614,44 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>https://cryptocurrencyjobs.co/design/oku-product-designer/</t>
+          <t>https://news.ycombinator.com/item?id=49922584</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Web3, Blockchain, Crypto</t>
+          <t>Tech, Startup, Engineering</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:13.007399+00:00</t>
+          <t>2026-10-21T08:15:38.528497+00:00</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CryptoJobs</t>
+          <t>CryptoCurrencyJobs</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>SRC-0075</t>
+          <t>SRC-0073</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Web3 DApp Developer (Remote)</t>
+          <t>Senior Software Engineer - Compiler</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>spinbattles</t>
+          <t>Category Labs</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Global / Remote</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -4681,44 +4673,44 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>https://www.cryptojobs.com/job/web3-dapp-developer-remote-12463</t>
+          <t>https://cryptocurrencyjobs.co/engineering/category-labs-senior-software-engineer-compiler/</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>Web3, Blockchain, Solidity, Crypto</t>
+          <t>Web3, Blockchain, Crypto</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:17.378987+00:00</t>
+          <t>2026-10-21T08:15:39.303464+00:00</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CryptoJobs</t>
+          <t>CryptoCurrencyJobs</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SRC-0075</t>
+          <t>SRC-0073</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>DevSecOps Engineer</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>RWAHub</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Global / Remote</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -4740,44 +4732,44 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>https://www.cryptojobs.com/job/backend-engineer-12459</t>
+          <t>https://cryptocurrencyjobs.co/engineering/casa-devsecops-engineer/</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Web3, Blockchain, Solidity, Crypto</t>
+          <t>Web3, Blockchain, Crypto</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:17.379987+00:00</t>
+          <t>2026-10-21T08:15:39.303464+00:00</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>WWRDevOps</t>
+          <t>CryptoJobs</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SRC-0041</t>
+          <t>SRC-0075</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Customer Solutions Engineer, EMEA</t>
+          <t>Web3 DApp Developer (Remote)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>spinbattles</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Global / Remote</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -4799,44 +4791,44 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-customer-solutions-engineer-emea</t>
+          <t>https://www.cryptojobs.com/job/web3-dapp-developer-remote-12463</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>DevOps, SysAdmin, Cloud, Infrastructure, Kubernetes</t>
+          <t>Web3, Blockchain, Solidity, Crypto</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:18.748083+00:00</t>
+          <t>2026-10-21T08:15:40.681811+00:00</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>WWRDevOps</t>
+          <t>CryptoJobs</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SRC-0041</t>
+          <t>SRC-0075</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Sales Development Representative - Service Provider</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Huntress</t>
+          <t>RWAHub</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Global / Remote</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -4858,39 +4850,39 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/huntress-sales-development-representative-service-provider</t>
+          <t>https://www.cryptojobs.com/job/backend-engineer-12459</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>DevOps, SysAdmin, Cloud, Infrastructure, Kubernetes</t>
+          <t>Web3, Blockchain, Solidity, Crypto</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:18.748083+00:00</t>
+          <t>2026-10-21T08:15:40.681811+00:00</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>WWRProduct</t>
+          <t>WWRDevOps</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SRC-0045</t>
+          <t>SRC-0041</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Lead Product Manager</t>
+          <t>Director, Information Security</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Lattice</t>
+          <t>Carrot</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4917,39 +4909,39 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/lattice-lead-product-manager</t>
+          <t>https://weworkremotely.com/remote-jobs/carrot-director-information-security</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Product Management, Product Strategy, Agile, Scrum</t>
+          <t>DevOps, SysAdmin, Cloud, Infrastructure, Kubernetes</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:20.046276+00:00</t>
+          <t>2026-10-21T08:15:41.324373+00:00</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>WWRProduct</t>
+          <t>WWRDevOps</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SRC-0045</t>
+          <t>SRC-0041</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Principal Product Manager, Savings (R13997)</t>
+          <t>Senior Security Engineer, Detection &amp; Response</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Oportun</t>
+          <t>Flexport</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4976,44 +4968,44 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/oportun-principal-product-manager-savings-r13997</t>
+          <t>https://weworkremotely.com/remote-jobs/flexport-senior-security-engineer-detection-response</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>Product Management, Product Strategy, Agile, Scrum</t>
+          <t>DevOps, SysAdmin, Cloud, Infrastructure, Kubernetes</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:20.046276+00:00</t>
+          <t>2026-10-21T08:15:41.324373+00:00</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>RemoteOKEngineer</t>
+          <t>WWRProduct</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SRC-0050</t>
+          <t>SRC-0045</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Principal Product Manager Strategic Initiatives</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Thyme Care</t>
+          <t>Upsun</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Global / Remote</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -5028,47 +5020,51 @@
       </c>
       <c r="H80" t="inlineStr"/>
       <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-principal-product-manager-strategic-initiatives-thyme-care-1137510</t>
+          <t>https://weworkremotely.com/remote-jobs/upsun-product-manager</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>product manager, exec, technical, customer support, testing, senior, ops, medical</t>
+          <t>Product Management, Product Strategy, Agile, Scrum</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:21.157231+00:00</t>
+          <t>2026-10-21T08:15:43.795695+00:00</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>RemoteOKEngineer</t>
+          <t>WWRProduct</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SRC-0050</t>
+          <t>SRC-0045</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Principal Software Engineer</t>
+          <t>Manager II, Developer Advocacy</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Vytalize Health</t>
+          <t>Datadog</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>Global / Remote</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -5083,20 +5079,134 @@
       </c>
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-principal-software-engineer-vytalize-health-1137508</t>
+          <t>https://weworkremotely.com/remote-jobs/datadog-manager-ii-developer-advocacy</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>dev, design, infosec, python, docker, technical, recruiter, customer support</t>
+          <t>Product Management, Product Strategy, Agile, Scrum</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>2026-10-16T07:26:21.157231+00:00</t>
+          <t>2026-10-21T08:15:43.795695+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>RemoteOKEngineer</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>SRC-0050</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Sothebyâs</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Worldwide / Remote</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-senior-software-engineer-sothebys-1137545</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>golang, dev, senior, sales, engineer, digital nomad</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>2026-10-21T08:15:44.703898+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>RemoteOKEngineer</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>SRC-0050</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Senior Backend Engineer</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Rain</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Worldwide / Remote</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-senior-backend-engineer-rain-1137544</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>golang, finance, mobile, senior, medical, engineer, backend</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>2026-10-21T08:15:44.704907+00:00</t>
         </is>
       </c>
     </row>
@@ -5504,16 +5614,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Careerjet</t>
+          <t>Careerjet India</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>NO_DATA</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -5544,7 +5654,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cutshort</t>
+          <t>Cutshort Tech &amp; AI</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -5604,7 +5714,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Jobsora</t>
+          <t>Jobsora Aggregator</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -5624,7 +5734,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PlacementIndia</t>
+          <t>Placement India</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">

</xml_diff>